<commit_message>
fix(ui): refactor virtual scrolling to use IntersectionObserver
- Replaced mathematical scroll offset logic with a sentinel `IntersectionObserver` in `DataTable` to resolve infinite loading loops and missing initial loads.
- Made `nextPage` optional in `PaginationResponse` type, mapping undefined returns correctly across all paginated entities (Users, Exams, Students, Activities).
- Created a `hasPermission` server utility to handle auth redirects consistently and cleaned up `UsersPage` permission checks.
- Fixed schema typing for missing parameters like `studentId` string casting and null `rut` properties.
</commit_message>
<xml_diff>
--- a/prisma/data/estructura_bd.xlsx
+++ b/prisma/data/estructura_bd.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE2063F-B5B5-4E52-96AB-65765A2444E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📌 Índice" sheetId="1" r:id="rId1"/>
@@ -2358,20 +2358,20 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2397,6 +2397,83 @@
         <bottom style="thin">
           <color rgb="FFAAAAAA"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFAAAAAA"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFAAAAAA"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAAAAAA"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAAAAAA"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAAAAAA"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAAAAAA"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAAAAAA"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2426,7 +2503,50 @@
         <left style="thin">
           <color rgb="FFAAAAAA"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color rgb="FFAAAAAA"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAAAAAA"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAAAAAA"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAAAAAA"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAAAAAA"/>
+        </right>
         <top style="thin">
           <color rgb="FFAAAAAA"/>
         </top>
@@ -2500,7 +2620,44 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFAAAAAA"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAAAAAA"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAAAAAA"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FFAAAAAA"/>
         </left>
@@ -2513,8 +2670,6 @@
         <bottom style="thin">
           <color rgb="FFAAAAAA"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2540,61 +2695,17 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FFAAAAAA"/>
         </left>
-        <right style="thin">
-          <color rgb="FFAAAAAA"/>
-        </right>
+        <right/>
         <top style="thin">
           <color rgb="FFAAAAAA"/>
         </top>
         <bottom style="thin">
           <color rgb="FFAAAAAA"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFAAAAAA"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFAAAAAA"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFAAAAAA"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFAAAAAA"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -5515,51 +5626,12 @@
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFAAAAAA"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFAAAAAA"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFAAAAAA"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color rgb="FFAAAAAA"/>
         </left>
-        <right style="thin">
-          <color rgb="FFAAAAAA"/>
-        </right>
+        <right/>
         <top style="thin">
           <color rgb="FFAAAAAA"/>
         </top>
@@ -5626,7 +5698,6 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -5714,8 +5785,10 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAAAAAA"/>
+        </left>
         <right style="thin">
           <color rgb="FFAAAAAA"/>
         </right>
@@ -5725,81 +5798,8 @@
         <bottom style="thin">
           <color rgb="FFAAAAAA"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFAAAAAA"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFAAAAAA"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFAAAAAA"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFAAAAAA"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFAAAAAA"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFAAAAAA"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFAAAAAA"/>
-        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -5971,58 +5971,58 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{21BDF646-6AB5-43B7-AD3B-7DFA6765727B}" name="ADegreeTable" displayName="ADegreeTable" ref="A6:B8" totalsRowShown="0" headerRowDxfId="105" headerRowBorderDxfId="104" tableBorderDxfId="103" totalsRowBorderDxfId="102">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{21BDF646-6AB5-43B7-AD3B-7DFA6765727B}" name="ADegreeTable" displayName="ADegreeTable" ref="A6:B8" totalsRowShown="0" headerRowDxfId="108" headerRowBorderDxfId="107" tableBorderDxfId="106" totalsRowBorderDxfId="105">
   <autoFilter ref="A6:B8" xr:uid="{21BDF646-6AB5-43B7-AD3B-7DFA6765727B}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D084344C-E421-48F0-8ED9-9638F88C6846}" name="id"/>
-    <tableColumn id="2" xr3:uid="{9F0DCB94-4F04-48E3-B0C1-197AD7B74B6B}" name="name" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{9F0DCB94-4F04-48E3-B0C1-197AD7B74B6B}" name="name" dataDxfId="104"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7B666A61-9D82-4C49-BCCD-2E916244936B}" name="TemplateTable" displayName="TemplateTable" ref="A6:I11" totalsRowShown="0" headerRowDxfId="119" dataDxfId="117" headerRowBorderDxfId="118" tableBorderDxfId="116" totalsRowBorderDxfId="115">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7B666A61-9D82-4C49-BCCD-2E916244936B}" name="TemplateTable" displayName="TemplateTable" ref="A6:I11" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12">
   <autoFilter ref="A6:I11" xr:uid="{7B666A61-9D82-4C49-BCCD-2E916244936B}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{35DFD295-E223-4974-ACE2-697935223713}" name="id" dataDxfId="114">
+    <tableColumn id="1" xr3:uid="{35DFD295-E223-4974-ACE2-697935223713}" name="id" dataDxfId="11">
       <calculatedColumnFormula>IF(ISBLANK(TemplateTable[[#This Row],[certificateName]]),"",ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F0014E9D-997A-4846-891A-BB433D709D81}" name="certificateName" dataDxfId="113"/>
-    <tableColumn id="3" xr3:uid="{6800626F-D286-415C-A674-0DB3C1DB73C2}" name="certificateId" dataDxfId="112">
+    <tableColumn id="2" xr3:uid="{F0014E9D-997A-4846-891A-BB433D709D81}" name="certificateName" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{6800626F-D286-415C-A674-0DB3C1DB73C2}" name="certificateId" dataDxfId="9">
       <calculatedColumnFormula>_xlfn.XLOOKUP(TemplateTable[[#This Row],[certificateName]],CertificateTable[name], CertificateTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{98120E82-B208-4584-AA36-331D4263F344}" name="role" dataDxfId="111"/>
-    <tableColumn id="8" xr3:uid="{1EC5D45E-1355-4169-9B29-F2DD20E04EC2}" name="activityTypeName" dataDxfId="110"/>
-    <tableColumn id="5" xr3:uid="{BFE3FA6C-D650-450B-9013-3E601CEFEAB9}" name="activityTypeId" dataDxfId="109">
+    <tableColumn id="4" xr3:uid="{98120E82-B208-4584-AA36-331D4263F344}" name="role" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{1EC5D45E-1355-4169-9B29-F2DD20E04EC2}" name="activityTypeName" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{BFE3FA6C-D650-450B-9013-3E601CEFEAB9}" name="activityTypeId" dataDxfId="6">
       <calculatedColumnFormula>_xlfn.XLOOKUP(TemplateTable[[#This Row],[activityTypeName]], ActivityTypeTable[name],ActivityTypeTable[id], "",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{D2A34400-809B-4181-B7DE-643FA4E237AC}" name="participantTypeName" dataDxfId="108"/>
-    <tableColumn id="6" xr3:uid="{C114DF71-6DF2-480D-932F-564F087EDE4D}" name="participantTypeId" dataDxfId="107">
+    <tableColumn id="9" xr3:uid="{D2A34400-809B-4181-B7DE-643FA4E237AC}" name="participantTypeName" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{C114DF71-6DF2-480D-932F-564F087EDE4D}" name="participantTypeId" dataDxfId="4">
       <calculatedColumnFormula>_xlfn.XLOOKUP(TemplateTable[[#This Row],[participantTypeName]], ParticipantTypeTable[name], ParticipantTypeTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{718F385C-1FA2-47C7-A2A8-851AF99822CD}" name="template" dataDxfId="106"/>
+    <tableColumn id="7" xr3:uid="{718F385C-1FA2-47C7-A2A8-851AF99822CD}" name="template" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BC5C6D74-FC52-47E2-AA34-D6697409B949}" name="ExamTable" displayName="ExamTable" ref="A6:F7" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BC5C6D74-FC52-47E2-AA34-D6697409B949}" name="ExamTable" displayName="ExamTable" ref="A6:F7" totalsRowShown="0" headerRowDxfId="119" dataDxfId="117" headerRowBorderDxfId="118" tableBorderDxfId="116" totalsRowBorderDxfId="115">
   <autoFilter ref="A6:F7" xr:uid="{BC5C6D74-FC52-47E2-AA34-D6697409B949}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{692719ED-79B2-42F7-9EE5-149A32F745B3}" name="id" dataDxfId="8">
+    <tableColumn id="1" xr3:uid="{692719ED-79B2-42F7-9EE5-149A32F745B3}" name="id" dataDxfId="114">
       <calculatedColumnFormula>IF(ISBLANK(ExamTable[[#This Row],[studentName]]),"",ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1B246D39-0161-43B5-A25E-5F63C4AE1C13}" name="studentName" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{9CA5A4E7-4070-4BCC-8ABE-22A888226F06}" name="activityName" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{21CCAFCC-797A-43FF-B871-B5CE4FD3B169}" name="studentId" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{1B246D39-0161-43B5-A25E-5F63C4AE1C13}" name="studentName" dataDxfId="113"/>
+    <tableColumn id="3" xr3:uid="{9CA5A4E7-4070-4BCC-8ABE-22A888226F06}" name="activityName" dataDxfId="112"/>
+    <tableColumn id="4" xr3:uid="{21CCAFCC-797A-43FF-B871-B5CE4FD3B169}" name="studentId" dataDxfId="111">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ExamTable[[#This Row],[studentName]],StudentTable[userName],StudentTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{6E4D44FF-C970-45A8-9C7A-5AE471194553}" name="activityId" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{6E4D44FF-C970-45A8-9C7A-5AE471194553}" name="activityId" dataDxfId="110">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ExamTable[[#This Row],[activityName]],ActivityTable[name], ActivityTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{9C8DA54A-7DAD-473A-A016-641BD60DCBEA}" name="grade" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{9C8DA54A-7DAD-473A-A016-641BD60DCBEA}" name="grade" dataDxfId="109"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6048,41 +6048,41 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D06504D-941D-4F95-A34D-8031062A23F0}" name="TitleTable" displayName="TitleTable" ref="A6:E12" totalsRowShown="0" headerRowDxfId="100" headerRowBorderDxfId="99" tableBorderDxfId="98" totalsRowBorderDxfId="97">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D06504D-941D-4F95-A34D-8031062A23F0}" name="TitleTable" displayName="TitleTable" ref="A6:E12" totalsRowShown="0" headerRowDxfId="103" headerRowBorderDxfId="102" tableBorderDxfId="101" totalsRowBorderDxfId="100">
   <autoFilter ref="A6:E12" xr:uid="{1D06504D-941D-4F95-A34D-8031062A23F0}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7801D28A-9FC1-4168-B38F-EE639910650A}" name="id" dataDxfId="96">
+    <tableColumn id="1" xr3:uid="{7801D28A-9FC1-4168-B38F-EE639910650A}" name="id" dataDxfId="99">
       <calculatedColumnFormula>IF(TitleTable[[#This Row],[academicDegreeId]]&lt;&gt;"",ROW()-6,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A7BC7DF6-3102-4BBA-BC51-DB8410EAB5BD}" name="academicDegreeId" dataDxfId="95">
+    <tableColumn id="2" xr3:uid="{A7BC7DF6-3102-4BBA-BC51-DB8410EAB5BD}" name="academicDegreeId" dataDxfId="98">
       <calculatedColumnFormula>_xlfn.XLOOKUP(TitleTable[[#This Row],[AcademicDegreeName]],ADegreeTable[name], ADegreeTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A4F7459D-7F69-4F60-BB9E-B23C34251DCF}" name="AcademicDegreeName" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{300E313B-FA95-4376-9612-7FF1A398FA49}" name="gender" dataDxfId="93"/>
-    <tableColumn id="4" xr3:uid="{30F0397B-1916-4C7E-B449-91C6BCF48ADA}" name="abbrev" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{A4F7459D-7F69-4F60-BB9E-B23C34251DCF}" name="AcademicDegreeName" dataDxfId="97"/>
+    <tableColumn id="3" xr3:uid="{300E313B-FA95-4376-9612-7FF1A398FA49}" name="gender" dataDxfId="96"/>
+    <tableColumn id="4" xr3:uid="{30F0397B-1916-4C7E-B449-91C6BCF48ADA}" name="abbrev" dataDxfId="95"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{85FEA289-536E-4259-A619-2744ADA3DB87}" name="UserTable" displayName="UserTable" ref="A6:N36" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90" tableBorderDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{85FEA289-536E-4259-A619-2744ADA3DB87}" name="UserTable" displayName="UserTable" ref="A6:N36" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93" tableBorderDxfId="92">
   <autoFilter ref="A6:N36" xr:uid="{85FEA289-536E-4259-A619-2744ADA3DB87}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{D84565A3-15A3-40D5-885B-59C4991B2454}" name="id" dataDxfId="88">
+    <tableColumn id="1" xr3:uid="{D84565A3-15A3-40D5-885B-59C4991B2454}" name="id" dataDxfId="91">
       <calculatedColumnFormula>IF(UserTable[[#This Row],[rut]]&lt;&gt;"", ROW()-6,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E789B167-226C-420B-BBD4-8755387CAFE6}" name="rut" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{93B4A9A1-DC9A-44FA-8692-C9A24CC1BF40}" name="name" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{63AB093F-B349-4655-86C2-B260E78F6BF1}" name="email" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{56D0A7C0-F001-4955-A153-E7F45CC5AF52}" name="emailVerified" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{7D04D1EC-A119-48D6-AD1F-240337054887}" name="image" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{CF3A91BB-659C-4083-935E-AFC637FBA3F3}" name="role" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{5C06DE85-13EF-4A5C-B6DB-B75E5FFC0545}" name="banned" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{8BFEF23D-7870-4777-A520-8246B3DE2FDF}" name="banReason" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{F672B4C8-D389-49C1-9B64-DE4E88445A59}" name="banExpires" dataDxfId="79"/>
-    <tableColumn id="11" xr3:uid="{90307C6C-1290-4627-8E69-FF7293A360C8}" name="gender" dataDxfId="78"/>
-    <tableColumn id="12" xr3:uid="{AFFA8672-1495-4235-9B93-04970AC93F2A}" name="isDirector" dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{E789B167-226C-420B-BBD4-8755387CAFE6}" name="rut" dataDxfId="90"/>
+    <tableColumn id="3" xr3:uid="{93B4A9A1-DC9A-44FA-8692-C9A24CC1BF40}" name="name" dataDxfId="89"/>
+    <tableColumn id="4" xr3:uid="{63AB093F-B349-4655-86C2-B260E78F6BF1}" name="email" dataDxfId="88"/>
+    <tableColumn id="5" xr3:uid="{56D0A7C0-F001-4955-A153-E7F45CC5AF52}" name="emailVerified" dataDxfId="87"/>
+    <tableColumn id="6" xr3:uid="{7D04D1EC-A119-48D6-AD1F-240337054887}" name="image" dataDxfId="86"/>
+    <tableColumn id="7" xr3:uid="{CF3A91BB-659C-4083-935E-AFC637FBA3F3}" name="role" dataDxfId="85"/>
+    <tableColumn id="8" xr3:uid="{5C06DE85-13EF-4A5C-B6DB-B75E5FFC0545}" name="banned" dataDxfId="84"/>
+    <tableColumn id="9" xr3:uid="{8BFEF23D-7870-4777-A520-8246B3DE2FDF}" name="banReason" dataDxfId="83"/>
+    <tableColumn id="10" xr3:uid="{F672B4C8-D389-49C1-9B64-DE4E88445A59}" name="banExpires" dataDxfId="82"/>
+    <tableColumn id="11" xr3:uid="{90307C6C-1290-4627-8E69-FF7293A360C8}" name="gender" dataDxfId="81"/>
+    <tableColumn id="12" xr3:uid="{AFFA8672-1495-4235-9B93-04970AC93F2A}" name="isDirector" dataDxfId="80"/>
     <tableColumn id="13" xr3:uid="{623D3833-0700-46BB-9F79-F1EBAFC81D6A}" name="academicDegreeId">
       <calculatedColumnFormula>_xlfn.XLOOKUP(UserTable[[#This Row],[academicDegreeName]], ADegreeTable[name], ADegreeTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
@@ -6093,111 +6093,111 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FCF25C97-1CFC-458F-A99C-18D9A6AD8A69}" name="StudentTable" displayName="StudentTable" ref="A6:F31" totalsRowShown="0" headerRowDxfId="76" dataDxfId="74" headerRowBorderDxfId="75" tableBorderDxfId="73" totalsRowBorderDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FCF25C97-1CFC-458F-A99C-18D9A6AD8A69}" name="StudentTable" displayName="StudentTable" ref="A6:F31" totalsRowShown="0" headerRowDxfId="79" dataDxfId="77" headerRowBorderDxfId="78" tableBorderDxfId="76" totalsRowBorderDxfId="75">
   <autoFilter ref="A6:F31" xr:uid="{FCF25C97-1CFC-458F-A99C-18D9A6AD8A69}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{4365B9E5-05D3-43F2-9E75-34DB73C72A3F}" name="id" dataDxfId="71">
+    <tableColumn id="1" xr3:uid="{4365B9E5-05D3-43F2-9E75-34DB73C72A3F}" name="id" dataDxfId="74">
       <calculatedColumnFormula>IF(ISBLANK(StudentTable[[#This Row],[studentId]]),"", ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EAC8744D-1F09-4A5C-8E4A-3D85E08B6D37}" name="studentId" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{66B37519-AF27-4C0F-9BFE-4DE89E499C64}" name="userName" dataDxfId="69"/>
-    <tableColumn id="4" xr3:uid="{76391975-9083-4AF9-B31F-55AE28819CFB}" name="userId" dataDxfId="68">
+    <tableColumn id="2" xr3:uid="{EAC8744D-1F09-4A5C-8E4A-3D85E08B6D37}" name="studentId" dataDxfId="73"/>
+    <tableColumn id="3" xr3:uid="{66B37519-AF27-4C0F-9BFE-4DE89E499C64}" name="userName" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{76391975-9083-4AF9-B31F-55AE28819CFB}" name="userId" dataDxfId="71">
       <calculatedColumnFormula>_xlfn.XLOOKUP(StudentTable[[#This Row],[userName]],UserTable[name],UserTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{BD538411-70FF-493E-B572-8105AB255D28}" name="isRegularStudent" dataDxfId="67"/>
-    <tableColumn id="6" xr3:uid="{D2EBA512-F8A8-4CB6-8EA2-A0DC38CB5C0B}" name="admisionDate" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{BD538411-70FF-493E-B572-8105AB255D28}" name="isRegularStudent" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{D2EBA512-F8A8-4CB6-8EA2-A0DC38CB5C0B}" name="admisionDate" dataDxfId="69"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0F547C4C-61C7-4C2A-9C4D-C8523461AAFF}" name="ActivityTypeTable" displayName="ActivityTypeTable" ref="A6:B13" totalsRowShown="0" headerRowDxfId="65" headerRowBorderDxfId="64" tableBorderDxfId="63" totalsRowBorderDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0F547C4C-61C7-4C2A-9C4D-C8523461AAFF}" name="ActivityTypeTable" displayName="ActivityTypeTable" ref="A6:B13" totalsRowShown="0" headerRowDxfId="68" headerRowBorderDxfId="67" tableBorderDxfId="66" totalsRowBorderDxfId="65">
   <autoFilter ref="A6:B13" xr:uid="{0F547C4C-61C7-4C2A-9C4D-C8523461AAFF}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{59150BA5-A7DE-4874-BEC8-662316686ECE}" name="id" dataDxfId="61">
+    <tableColumn id="1" xr3:uid="{59150BA5-A7DE-4874-BEC8-662316686ECE}" name="id" dataDxfId="64">
       <calculatedColumnFormula>IF(ISBLANK(ActivityTypeTable[[#This Row],[name]]),"", ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C734BFB6-8090-4FE5-B857-573748EB0614}" name="name" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{C734BFB6-8090-4FE5-B857-573748EB0614}" name="name" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DF67C1A1-6942-4B9F-AE16-A9B361C53B1A}" name="ActivityTable" displayName="ActivityTable" ref="A6:H7" totalsRowShown="0" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56" totalsRowBorderDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DF67C1A1-6942-4B9F-AE16-A9B361C53B1A}" name="ActivityTable" displayName="ActivityTable" ref="A6:H7" totalsRowShown="0" headerRowDxfId="62" dataDxfId="60" headerRowBorderDxfId="61" tableBorderDxfId="59" totalsRowBorderDxfId="58">
   <autoFilter ref="A6:H7" xr:uid="{DF67C1A1-6942-4B9F-AE16-A9B361C53B1A}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{ED578E86-4E76-4E90-85CA-674930C235F7}" name="id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{FB6C5FA6-DF04-45A7-89B5-88F1FC79C2D6}" name="activityTypeName" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{EE938535-FAD5-46E2-9062-D0D81D92843E}" name="activityTypeId" dataDxfId="52">
+    <tableColumn id="1" xr3:uid="{ED578E86-4E76-4E90-85CA-674930C235F7}" name="id" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{FB6C5FA6-DF04-45A7-89B5-88F1FC79C2D6}" name="activityTypeName" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{EE938535-FAD5-46E2-9062-D0D81D92843E}" name="activityTypeId" dataDxfId="55">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ActivityTable[[#This Row],[activityTypeName]],ActivityTypeTable[name], ActivityTypeTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7E99DBF1-B701-4269-8285-40CB77EE77CF}" name="name" dataDxfId="51"/>
-    <tableColumn id="5" xr3:uid="{3F2225E0-5303-4D1E-95EC-65F1B96512C6}" name="startAt" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{D19CBEFD-D71A-41F7-A14B-DF9F5A8E0CA5}" name="endAt" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{A77D4338-9AE4-4919-BC5C-02F7DEF383DE}" name="nAssistant" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{AB81B6E6-2917-4082-9767-BA28157B6C97}" name="nParticipant" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{7E99DBF1-B701-4269-8285-40CB77EE77CF}" name="name" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{3F2225E0-5303-4D1E-95EC-65F1B96512C6}" name="startAt" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{D19CBEFD-D71A-41F7-A14B-DF9F5A8E0CA5}" name="endAt" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{A77D4338-9AE4-4919-BC5C-02F7DEF383DE}" name="nAssistant" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{AB81B6E6-2917-4082-9767-BA28157B6C97}" name="nParticipant" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{23ADF508-CC90-4FBB-B8A6-80FFBB135690}" name="ParticipantTypeTable" displayName="ParticipantTypeTable" ref="A6:G22" totalsRowShown="0" headerRowDxfId="46" dataDxfId="44" headerRowBorderDxfId="45" tableBorderDxfId="43" totalsRowBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{23ADF508-CC90-4FBB-B8A6-80FFBB135690}" name="ParticipantTypeTable" displayName="ParticipantTypeTable" ref="A6:G22" totalsRowShown="0" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48" tableBorderDxfId="46" totalsRowBorderDxfId="45">
   <autoFilter ref="A6:G22" xr:uid="{23ADF508-CC90-4FBB-B8A6-80FFBB135690}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{10A749B4-38CA-4B67-A4C5-C561F90DDDE2}" name="id" dataDxfId="41">
+    <tableColumn id="1" xr3:uid="{10A749B4-38CA-4B67-A4C5-C561F90DDDE2}" name="id" dataDxfId="44">
       <calculatedColumnFormula>IF(ISBLANK(ParticipantTypeTable[[#This Row],[name]]),"", ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{04AFB6EC-E691-421A-B26F-9891A42D291E}" name="name" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{12DF8505-E053-492C-8C45-4D52788AA007}" name="roles" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{D684A6E0-2CB6-43AD-AA2A-978621E5D4DB}" name="activityTypeName" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{8BB7BDF5-9C51-428B-8F41-2D5551800DA8}" name="activityTypeId" dataDxfId="37">
+    <tableColumn id="2" xr3:uid="{04AFB6EC-E691-421A-B26F-9891A42D291E}" name="name" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{12DF8505-E053-492C-8C45-4D52788AA007}" name="roles" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{D684A6E0-2CB6-43AD-AA2A-978621E5D4DB}" name="activityTypeName" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{8BB7BDF5-9C51-428B-8F41-2D5551800DA8}" name="activityTypeId" dataDxfId="40">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ParticipantTypeTable[[#This Row],[activityTypeName]],ActivityTypeTable[name], ActivityTypeTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D21DFADD-72C9-48EF-9B97-94DCE941715E}" name=" min" dataDxfId="36"/>
-    <tableColumn id="9" xr3:uid="{2EB78418-4933-4BE7-848D-737A5AED6CD7}" name="max" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{D21DFADD-72C9-48EF-9B97-94DCE941715E}" name=" min" dataDxfId="39"/>
+    <tableColumn id="9" xr3:uid="{2EB78418-4933-4BE7-848D-737A5AED6CD7}" name="max" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{15FD7229-441E-4FE3-AF45-908EA33D6E1A}" name="ParticipantTable" displayName="ParticipantTable" ref="A6:J7" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{15FD7229-441E-4FE3-AF45-908EA33D6E1A}" name="ParticipantTable" displayName="ParticipantTable" ref="A6:J7" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34" totalsRowBorderDxfId="33">
   <autoFilter ref="A6:J7" xr:uid="{15FD7229-441E-4FE3-AF45-908EA33D6E1A}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{652686EA-7035-4724-9CDA-D89B37DDB77D}" name="id" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{652686EA-7035-4724-9CDA-D89B37DDB77D}" name="id" dataDxfId="32">
       <calculatedColumnFormula>IF(ISBLANK(ParticipantTable[[#This Row],[activityName]]),"", ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{394ADFAF-FF0E-462F-BF79-96D9AFAC3CEA}" name="activityName" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{8FD18E64-E7FA-44AD-A7EC-413A12C07581}" name="userName" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{343F771A-82D0-4DC1-900F-370A7B1BECD0}" name="participantTypeName" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{BE01A539-C086-41E4-9971-BA82DB1D694F}" name="activityId" dataDxfId="25">
+    <tableColumn id="2" xr3:uid="{394ADFAF-FF0E-462F-BF79-96D9AFAC3CEA}" name="activityName" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{8FD18E64-E7FA-44AD-A7EC-413A12C07581}" name="userName" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{343F771A-82D0-4DC1-900F-370A7B1BECD0}" name="participantTypeName" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{BE01A539-C086-41E4-9971-BA82DB1D694F}" name="activityId" dataDxfId="28">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ParticipantTable[[#This Row],[activityName]],ActivityTable[name], ActivityTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0A7CDBA9-FD84-4CC8-8EDF-CD8D694398A9}" name="userId" dataDxfId="24">
+    <tableColumn id="6" xr3:uid="{0A7CDBA9-FD84-4CC8-8EDF-CD8D694398A9}" name="userId" dataDxfId="27">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ParticipantTable[[#This Row],[userName]],UserTable[name],UserTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F6E3050B-3F30-48C9-AAC7-FCAD98900424}" name="participantTypeId" dataDxfId="23">
+    <tableColumn id="7" xr3:uid="{F6E3050B-3F30-48C9-AAC7-FCAD98900424}" name="participantTypeId" dataDxfId="26">
       <calculatedColumnFormula>_xlfn.XLOOKUP(ParticipantTable[[#This Row],[participantTypeName]],ParticipantTypeTable[name],ParticipantTypeTable[id],"",0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{DACCFE94-858F-47FE-B4F6-B33E5374D14F}" name="hours" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{896BC859-D635-4695-B906-023A1E5FE6E6}" name="startAt" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{DFC6A317-6999-46F4-8CCD-ACD83FFB9F5E}" name="endAt" dataDxfId="20"/>
+    <tableColumn id="8" xr3:uid="{DACCFE94-858F-47FE-B4F6-B33E5374D14F}" name="hours" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{896BC859-D635-4695-B906-023A1E5FE6E6}" name="startAt" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{DFC6A317-6999-46F4-8CCD-ACD83FFB9F5E}" name="endAt" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{E4DFEBB4-E470-43F4-9B57-CA71A40CB7EA}" name="CertificateTable" displayName="CertificateTable" ref="A6:B13" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{E4DFEBB4-E470-43F4-9B57-CA71A40CB7EA}" name="CertificateTable" displayName="CertificateTable" ref="A6:B13" totalsRowShown="0" headerRowDxfId="22" headerRowBorderDxfId="21" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A6:B13" xr:uid="{E4DFEBB4-E470-43F4-9B57-CA71A40CB7EA}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{61038C46-43E9-4B35-96C1-CBBB1A87E834}" name="id" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{61038C46-43E9-4B35-96C1-CBBB1A87E834}" name="id" dataDxfId="18">
       <calculatedColumnFormula>IF(ISBLANK(CertificateTable[[#This Row],[name]]),"",ROW()-6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{33957B68-51D0-43D0-8BD3-562B4F9472E0}" name="name" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{33957B68-51D0-43D0-8BD3-562B4F9472E0}" name="name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6508,7 +6508,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="107" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="105"/>
@@ -6719,12 +6719,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>222</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
       <c r="E1" s="105"/>
       <c r="F1" s="105"/>
       <c r="G1" s="105"/>
@@ -6733,12 +6733,12 @@
       <c r="J1" s="105"/>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="104"/>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
       <c r="E2" s="105"/>
       <c r="F2" s="105"/>
       <c r="G2" s="105"/>
@@ -6939,13 +6939,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>238</v>
       </c>
       <c r="B1" s="105"/>
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>239</v>
       </c>
       <c r="B2" s="105"/>
@@ -7069,10 +7069,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>245</v>
       </c>
-      <c r="B1" s="107"/>
+      <c r="B1" s="109"/>
       <c r="C1" s="105"/>
       <c r="D1" s="105"/>
       <c r="E1" s="105"/>
@@ -7082,10 +7082,10 @@
       <c r="I1" s="105"/>
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>246</v>
       </c>
-      <c r="B2" s="104"/>
+      <c r="B2" s="106"/>
       <c r="C2" s="105"/>
       <c r="D2" s="105"/>
       <c r="E2" s="105"/>
@@ -7404,21 +7404,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>257</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
       <c r="D1" s="105"/>
       <c r="E1" s="105"/>
       <c r="F1" s="105"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>258</v>
       </c>
-      <c r="B2" s="104"/>
-      <c r="C2" s="104"/>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
       <c r="D2" s="105"/>
       <c r="E2" s="105"/>
       <c r="F2" s="105"/>
@@ -7565,7 +7565,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>265</v>
       </c>
       <c r="B1" s="105"/>
@@ -7576,7 +7576,7 @@
       <c r="G1" s="105"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>266</v>
       </c>
       <c r="B2" s="105"/>
@@ -7765,7 +7765,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="108" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="105"/>
@@ -7849,13 +7849,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="109" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="105"/>
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="105"/>
@@ -7939,7 +7939,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="109" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="105"/>
@@ -7948,7 +7948,7 @@
       <c r="E1" s="105"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>64</v>
       </c>
       <c r="B2" s="105"/>
@@ -8176,22 +8176,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
-      <c r="F1" s="106"/>
-      <c r="G1" s="106"/>
-      <c r="H1" s="106"/>
-      <c r="I1" s="106"/>
-      <c r="J1" s="106"/>
-      <c r="K1" s="106"/>
-      <c r="L1" s="106"/>
-      <c r="M1" s="106"/>
-      <c r="N1" s="106"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="110" t="s">
@@ -9417,7 +9417,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>158</v>
       </c>
       <c r="B1" s="105"/>
@@ -9427,7 +9427,7 @@
       <c r="F1" s="105"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>159</v>
       </c>
       <c r="B2" s="105"/>
@@ -10068,13 +10068,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>176</v>
       </c>
       <c r="B1" s="105"/>
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>177</v>
       </c>
       <c r="B2" s="105"/>
@@ -10195,10 +10195,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="107"/>
+      <c r="B1" s="109"/>
       <c r="C1" s="105"/>
       <c r="D1" s="105"/>
       <c r="E1" s="105"/>
@@ -10207,10 +10207,10 @@
       <c r="H1" s="105"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>187</v>
       </c>
-      <c r="B2" s="104"/>
+      <c r="B2" s="106"/>
       <c r="C2" s="105"/>
       <c r="D2" s="105"/>
       <c r="E2" s="105"/>
@@ -10411,7 +10411,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="104" t="s">
         <v>207</v>
       </c>
       <c r="B1" s="105"/>
@@ -10422,7 +10422,7 @@
       <c r="G1" s="105"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="106" t="s">
         <v>208</v>
       </c>
       <c r="B2" s="105"/>

</xml_diff>